<commit_message>
Finished PDF generation and print in all forms
</commit_message>
<xml_diff>
--- a/frontend/public/forms/templates/pc-template.xlsx
+++ b/frontend/public/forms/templates/pc-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GIO\Desktop\CHERIE\CAPSTONE\frontend\public\forms\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9F0067A-53CB-4D3C-A862-AB56F11515EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5428F979-41CE-43E4-9EBE-3ADC5E5D779D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Date</t>
   </si>
@@ -48,21 +48,12 @@
   </si>
   <si>
     <t>Remarks</t>
-  </si>
-  <si>
-    <t>Fund Cluster: ______________________</t>
   </si>
   <si>
     <t>Reference/
 PAR  No.</t>
   </si>
   <si>
-    <t>Property Number:_____________________</t>
-  </si>
-  <si>
-    <t>Entity Name : ________________________________________</t>
-  </si>
-  <si>
     <t>Property, Plant and Equipment :</t>
   </si>
   <si>
@@ -73,28 +64,34 @@
   </si>
   <si>
     <t>Appendix 69</t>
+  </si>
+  <si>
+    <t>Property Number:</t>
+  </si>
+  <si>
+    <t>Fund Cluster:</t>
+  </si>
+  <si>
+    <t>Entity Name :</t>
+  </si>
+  <si>
+    <t>Month:</t>
+  </si>
+  <si>
+    <t>PO #:</t>
+  </si>
+  <si>
+    <t>S/N:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <name val="Times New Roman"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
     </font>
     <font>
       <i/>
@@ -108,24 +105,7 @@
       <family val="1"/>
     </font>
     <font>
-      <sz val="14"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Times New Roman"/>
-      <family val="1"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="14"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -134,6 +114,51 @@
       <sz val="13"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -145,12 +170,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFCC00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -576,250 +601,255 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,6 +857,11 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFFCC00"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1302,389 +1337,404 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="2" width="10.59765625" customWidth="1"/>
+    <col min="2" max="2" width="16.59765625" customWidth="1"/>
     <col min="3" max="3" width="14.19921875" customWidth="1"/>
     <col min="4" max="5" width="10.59765625" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="17.5" customWidth="1"/>
     <col min="8" max="8" width="10.59765625" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="9" max="9" width="17.59765625" customWidth="1"/>
     <col min="10" max="10" width="19.8984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28">
+    <row r="1" spans="1:11" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="56">
         <v>169</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="38.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="56"/>
+      <c r="B2" s="65" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="67"/>
+    </row>
+    <row r="3" spans="1:11" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="56"/>
+      <c r="B3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="68"/>
+      <c r="F3" s="68"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="9"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="56"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="11"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="12"/>
+      <c r="J4" s="13"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="56"/>
+      <c r="B5" s="14" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="28"/>
-      <c r="J2" s="14"/>
-    </row>
-    <row r="3" spans="1:10" ht="33.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="28"/>
-      <c r="B3" s="38" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
-      <c r="H3" s="39"/>
-      <c r="I3" s="39"/>
-      <c r="J3" s="40"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="21"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
-      <c r="B5" s="22" t="s">
+      <c r="C5" s="69"/>
+      <c r="D5" s="69"/>
+      <c r="E5" s="69"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="16"/>
+      <c r="I5" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" s="17"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" ht="7.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="56"/>
+      <c r="B6" s="61"/>
+      <c r="C6" s="62"/>
+      <c r="D6" s="62"/>
+      <c r="E6" s="62"/>
+      <c r="F6" s="62"/>
+      <c r="G6" s="62"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="18"/>
+      <c r="J6" s="19"/>
+    </row>
+    <row r="7" spans="1:11" s="3" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="56"/>
+      <c r="B7" s="74" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="75"/>
+      <c r="D7" s="75"/>
+      <c r="E7" s="75"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="78"/>
+      <c r="I7" s="70" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="72"/>
+    </row>
+    <row r="8" spans="1:11" s="3" customFormat="1" ht="6.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="56"/>
+      <c r="B8" s="76"/>
+      <c r="C8" s="77"/>
+      <c r="D8" s="77"/>
+      <c r="E8" s="77"/>
+      <c r="F8" s="77"/>
+      <c r="G8" s="77"/>
+      <c r="H8" s="79"/>
+      <c r="I8" s="71"/>
+      <c r="J8" s="73"/>
+    </row>
+    <row r="9" spans="1:11" s="3" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="56"/>
+      <c r="B9" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9" s="21"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="60"/>
+      <c r="I9" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="J9" s="38"/>
+    </row>
+    <row r="10" spans="1:11" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="56"/>
+      <c r="B10" s="43" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" s="63" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="E10" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J5" s="23"/>
-    </row>
-    <row r="6" spans="1:10" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="28"/>
-      <c r="B6" s="46"/>
-      <c r="C6" s="47"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="24"/>
-      <c r="J6" s="25"/>
-    </row>
-    <row r="7" spans="1:10" s="8" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
-      <c r="B7" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" s="30"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="30"/>
-      <c r="H7" s="33"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="7"/>
-    </row>
-    <row r="8" spans="1:10" s="8" customFormat="1" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="28"/>
-      <c r="B8" s="31"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="34"/>
-      <c r="I8" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" s="10"/>
-    </row>
-    <row r="9" spans="1:10" s="8" customFormat="1" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="28"/>
-      <c r="B9" s="35" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="36"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="37"/>
-      <c r="I9" s="11"/>
-      <c r="J9" s="12"/>
-    </row>
-    <row r="10" spans="1:10" s="8" customFormat="1" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="28"/>
-      <c r="B10" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>5</v>
-      </c>
-      <c r="E10" s="41" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="42"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="13" t="s">
+      <c r="F10" s="48"/>
+      <c r="G10" s="49"/>
+      <c r="H10" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="I10" s="26" t="s">
+      <c r="I10" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="26" t="s">
+      <c r="J10" s="43" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="8" customFormat="1" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="28"/>
-      <c r="B11" s="27"/>
-      <c r="C11" s="49"/>
-      <c r="D11" s="16" t="s">
+    <row r="11" spans="1:11" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="56"/>
+      <c r="B11" s="44"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="F11" s="44" t="s">
+      <c r="F11" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="45"/>
-      <c r="H11" s="16" t="s">
+      <c r="G11" s="51"/>
+      <c r="H11" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="I11" s="27"/>
-      <c r="J11" s="27"/>
-    </row>
-    <row r="12" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
-      <c r="B12" s="70"/>
-      <c r="C12" s="58"/>
-      <c r="D12" s="58"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="50"/>
-      <c r="G12" s="51"/>
-      <c r="H12" s="58"/>
-      <c r="I12" s="60"/>
-      <c r="J12" s="60"/>
-    </row>
-    <row r="13" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="28"/>
-      <c r="B13" s="71"/>
-      <c r="C13" s="61"/>
-      <c r="D13" s="61"/>
-      <c r="E13" s="62"/>
-      <c r="F13" s="52"/>
-      <c r="G13" s="53"/>
-      <c r="H13" s="61"/>
-      <c r="I13" s="63"/>
-      <c r="J13" s="63"/>
-    </row>
-    <row r="14" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="28"/>
-      <c r="B14" s="71"/>
-      <c r="C14" s="61"/>
-      <c r="D14" s="61"/>
-      <c r="E14" s="62"/>
-      <c r="F14" s="52"/>
-      <c r="G14" s="53"/>
-      <c r="H14" s="61"/>
-      <c r="I14" s="63"/>
-      <c r="J14" s="63"/>
-    </row>
-    <row r="15" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="28"/>
-      <c r="B15" s="71"/>
-      <c r="C15" s="61"/>
-      <c r="D15" s="61"/>
-      <c r="E15" s="62"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="53"/>
-      <c r="H15" s="61"/>
-      <c r="I15" s="63"/>
-      <c r="J15" s="63"/>
-    </row>
-    <row r="16" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="28"/>
-      <c r="B16" s="71"/>
-      <c r="C16" s="61"/>
-      <c r="D16" s="61"/>
-      <c r="E16" s="62"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="53"/>
-      <c r="H16" s="61"/>
-      <c r="I16" s="63"/>
-      <c r="J16" s="63"/>
-    </row>
-    <row r="17" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="28"/>
-      <c r="B17" s="71"/>
-      <c r="C17" s="61"/>
-      <c r="D17" s="61"/>
-      <c r="E17" s="62"/>
-      <c r="F17" s="52"/>
-      <c r="G17" s="53"/>
-      <c r="H17" s="61"/>
-      <c r="I17" s="63"/>
-      <c r="J17" s="63"/>
-    </row>
-    <row r="18" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="28"/>
-      <c r="B18" s="71"/>
-      <c r="C18" s="61"/>
-      <c r="D18" s="61"/>
-      <c r="E18" s="62"/>
-      <c r="F18" s="52"/>
-      <c r="G18" s="53"/>
-      <c r="H18" s="61"/>
-      <c r="I18" s="63"/>
-      <c r="J18" s="63"/>
-    </row>
-    <row r="19" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="28"/>
-      <c r="B19" s="71"/>
-      <c r="C19" s="61"/>
-      <c r="D19" s="61"/>
-      <c r="E19" s="62"/>
-      <c r="F19" s="52"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="61"/>
-      <c r="I19" s="63"/>
-      <c r="J19" s="63"/>
-    </row>
-    <row r="20" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="28"/>
-      <c r="B20" s="71"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="62"/>
-      <c r="F20" s="52"/>
-      <c r="G20" s="53"/>
-      <c r="H20" s="61"/>
-      <c r="I20" s="63"/>
-      <c r="J20" s="63"/>
-    </row>
-    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="28"/>
-      <c r="B21" s="71"/>
-      <c r="C21" s="61"/>
-      <c r="D21" s="61"/>
-      <c r="E21" s="62"/>
-      <c r="F21" s="52"/>
-      <c r="G21" s="53"/>
-      <c r="H21" s="61"/>
-      <c r="I21" s="63"/>
-      <c r="J21" s="63"/>
-    </row>
-    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="28"/>
-      <c r="B22" s="72"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-      <c r="E22" s="65"/>
-      <c r="F22" s="52"/>
-      <c r="G22" s="53"/>
-      <c r="H22" s="64"/>
-      <c r="I22" s="66"/>
-      <c r="J22" s="66"/>
-    </row>
-    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="28"/>
-      <c r="B23" s="72"/>
-      <c r="C23" s="64"/>
-      <c r="D23" s="64"/>
-      <c r="E23" s="65"/>
-      <c r="F23" s="54"/>
-      <c r="G23" s="55"/>
-      <c r="H23" s="64"/>
-      <c r="I23" s="66"/>
-      <c r="J23" s="66"/>
-    </row>
-    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="28"/>
-      <c r="B24" s="72"/>
-      <c r="C24" s="64"/>
-      <c r="D24" s="64"/>
-      <c r="E24" s="65"/>
-      <c r="F24" s="54"/>
-      <c r="G24" s="55"/>
-      <c r="H24" s="64"/>
-      <c r="I24" s="66"/>
-      <c r="J24" s="66"/>
-    </row>
-    <row r="25" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="28"/>
-      <c r="B25" s="72"/>
-      <c r="C25" s="64"/>
-      <c r="D25" s="64"/>
-      <c r="E25" s="65"/>
-      <c r="F25" s="54"/>
-      <c r="G25" s="55"/>
-      <c r="H25" s="64"/>
-      <c r="I25" s="66"/>
-      <c r="J25" s="66"/>
-    </row>
-    <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28"/>
-      <c r="B26" s="72"/>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="65"/>
-      <c r="F26" s="54"/>
-      <c r="G26" s="55"/>
-      <c r="H26" s="64"/>
-      <c r="I26" s="66"/>
-      <c r="J26" s="66"/>
-    </row>
-    <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="28"/>
-      <c r="B27" s="72"/>
-      <c r="C27" s="64"/>
-      <c r="D27" s="64"/>
-      <c r="E27" s="65"/>
-      <c r="F27" s="54"/>
-      <c r="G27" s="55"/>
-      <c r="H27" s="64"/>
-      <c r="I27" s="66"/>
-      <c r="J27" s="66"/>
-    </row>
-    <row r="28" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="28"/>
-      <c r="B28" s="72"/>
-      <c r="C28" s="64"/>
-      <c r="D28" s="64"/>
-      <c r="E28" s="65"/>
-      <c r="F28" s="54"/>
-      <c r="G28" s="55"/>
-      <c r="H28" s="64"/>
-      <c r="I28" s="66"/>
-      <c r="J28" s="66"/>
-    </row>
-    <row r="29" spans="1:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="28"/>
-      <c r="B29" s="73"/>
-      <c r="C29" s="67"/>
-      <c r="D29" s="67"/>
-      <c r="E29" s="68"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="57"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="69"/>
-      <c r="J29" s="69"/>
+      <c r="I11" s="44"/>
+      <c r="J11" s="44"/>
+    </row>
+    <row r="12" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="56"/>
+      <c r="B12" s="25"/>
+      <c r="C12" s="25"/>
+      <c r="D12" s="25"/>
+      <c r="E12" s="26"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="53"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="27"/>
+    </row>
+    <row r="13" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="56"/>
+      <c r="B13" s="28"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
+      <c r="E13" s="29"/>
+      <c r="F13" s="54"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="40"/>
+      <c r="J13" s="30"/>
+    </row>
+    <row r="14" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="56"/>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="29"/>
+      <c r="F14" s="54"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="40"/>
+      <c r="J14" s="30"/>
+    </row>
+    <row r="15" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="56"/>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="29"/>
+      <c r="F15" s="54"/>
+      <c r="G15" s="55"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="40"/>
+      <c r="J15" s="30"/>
+    </row>
+    <row r="16" spans="1:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="56"/>
+      <c r="B16" s="28"/>
+      <c r="C16" s="28"/>
+      <c r="D16" s="28"/>
+      <c r="E16" s="29"/>
+      <c r="F16" s="54"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="40"/>
+      <c r="J16" s="30"/>
+    </row>
+    <row r="17" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="56"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="29"/>
+      <c r="F17" s="54"/>
+      <c r="G17" s="55"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="40"/>
+      <c r="J17" s="30"/>
+    </row>
+    <row r="18" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="56"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
+      <c r="E18" s="29"/>
+      <c r="F18" s="54"/>
+      <c r="G18" s="55"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="40"/>
+      <c r="J18" s="30"/>
+    </row>
+    <row r="19" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="56"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="54"/>
+      <c r="G19" s="55"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="40"/>
+      <c r="J19" s="30"/>
+    </row>
+    <row r="20" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="56"/>
+      <c r="B20" s="28"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="28"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="54"/>
+      <c r="G20" s="55"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="40"/>
+      <c r="J20" s="30"/>
+    </row>
+    <row r="21" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="56"/>
+      <c r="B21" s="28"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="28"/>
+      <c r="E21" s="29"/>
+      <c r="F21" s="54"/>
+      <c r="G21" s="55"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="40"/>
+      <c r="J21" s="30"/>
+    </row>
+    <row r="22" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="56"/>
+      <c r="B22" s="31"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="32"/>
+      <c r="F22" s="54"/>
+      <c r="G22" s="55"/>
+      <c r="H22" s="31"/>
+      <c r="I22" s="41"/>
+      <c r="J22" s="33"/>
+    </row>
+    <row r="23" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="56"/>
+      <c r="B23" s="31"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="31"/>
+      <c r="I23" s="41"/>
+      <c r="J23" s="33"/>
+    </row>
+    <row r="24" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="56"/>
+      <c r="B24" s="31"/>
+      <c r="C24" s="31"/>
+      <c r="D24" s="31"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="45"/>
+      <c r="G24" s="46"/>
+      <c r="H24" s="31"/>
+      <c r="I24" s="41"/>
+      <c r="J24" s="33"/>
+    </row>
+    <row r="25" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="56"/>
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="45"/>
+      <c r="G25" s="46"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="41"/>
+      <c r="J25" s="33"/>
+    </row>
+    <row r="26" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="56"/>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="32"/>
+      <c r="F26" s="45"/>
+      <c r="G26" s="46"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="41"/>
+      <c r="J26" s="33"/>
+    </row>
+    <row r="27" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="56"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="32"/>
+      <c r="F27" s="45"/>
+      <c r="G27" s="46"/>
+      <c r="H27" s="31"/>
+      <c r="I27" s="41"/>
+      <c r="J27" s="33"/>
+    </row>
+    <row r="28" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="56"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="45"/>
+      <c r="G28" s="46"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="41"/>
+      <c r="J28" s="33"/>
+    </row>
+    <row r="29" spans="1:10" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="56"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="35"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="58"/>
+      <c r="H29" s="34"/>
+      <c r="I29" s="42"/>
+      <c r="J29" s="36"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B30" s="1"/>
@@ -1693,17 +1743,34 @@
       <c r="B31" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="34">
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="I7:I8"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="B7:C8"/>
+    <mergeCell ref="D7:H8"/>
+    <mergeCell ref="A1:A29"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="D9:H9"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="F26:G26"/>
     <mergeCell ref="F27:G27"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="B2:J2"/>
     <mergeCell ref="J10:J11"/>
-    <mergeCell ref="B3:J3"/>
     <mergeCell ref="F25:G25"/>
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="F11:G11"/>
     <mergeCell ref="F12:G12"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="F24:G24"/>
     <mergeCell ref="F13:G13"/>
@@ -1711,20 +1778,6 @@
     <mergeCell ref="F15:G15"/>
     <mergeCell ref="I10:I11"/>
     <mergeCell ref="F22:G22"/>
-    <mergeCell ref="A1:A29"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="B7:D8"/>
-    <mergeCell ref="E7:H8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="F26:G26"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>